<commit_message>
BIDS update: changes to BlockInfo for info storage
</commit_message>
<xml_diff>
--- a/bids_functions/projectnameBIDS_BlockInfo.xlsx
+++ b/bids_functions/projectnameBIDS_BlockInfo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\serda\Documents\GitHub\CoreAdminCodes\bids_functions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B07A7A7-F244-422C-A513-36B42707250E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EADBAE5-8AC0-4D72-9D27-8246F6D17B1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="19">
   <si>
     <t>recording_info</t>
   </si>
@@ -33,15 +33,6 @@
     <t>comments</t>
   </si>
   <si>
-    <t>EEGDAT</t>
-  </si>
-  <si>
-    <t>ANALOGDATA</t>
-  </si>
-  <si>
-    <t>DIGITALDATA</t>
-  </si>
-  <si>
     <t>sub</t>
   </si>
   <si>
@@ -51,15 +42,6 @@
     <t>subject was fully attentive</t>
   </si>
   <si>
-    <t>data.streams.EEG1,data.streams.EEG2</t>
-  </si>
-  <si>
-    <t>data.streams.Wav8</t>
-  </si>
-  <si>
-    <t>data.epocs</t>
-  </si>
-  <si>
     <t>sub001</t>
   </si>
   <si>
@@ -78,13 +60,28 @@
     <t>auditoryLocalizer</t>
   </si>
   <si>
-    <t>edf</t>
-  </si>
-  <si>
-    <t>DC1,DC2</t>
-  </si>
-  <si>
-    <t>DC3</t>
+    <t>InstitutionAddress</t>
+  </si>
+  <si>
+    <t>Manufacturer</t>
+  </si>
+  <si>
+    <t>ManufacturersModelName</t>
+  </si>
+  <si>
+    <t>InstitutionName</t>
+  </si>
+  <si>
+    <t>UAB</t>
+  </si>
+  <si>
+    <t>1802 6th Avenue South, Birmingham, AL 35233</t>
+  </si>
+  <si>
+    <t>Natus</t>
+  </si>
+  <si>
+    <t>Unknown</t>
   </si>
 </sst>
 </file>
@@ -539,32 +536,34 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AMJ3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="8" style="1" customWidth="1"/>
-    <col min="3" max="3" width="11" style="1" customWidth="1"/>
-    <col min="4" max="4" width="10.5546875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="26.5546875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="26.6640625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="40.44140625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="20.44140625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="15.77734375" style="1" customWidth="1"/>
-    <col min="10" max="1024" width="11.5546875" style="1"/>
-    <col min="1025" max="1026" width="11.5546875"/>
+    <col min="1" max="1" width="8.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="49.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="28" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="1024" width="11.5703125" style="1"/>
+    <col min="1025" max="1026" width="11.5703125"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>0</v>
@@ -573,76 +572,86 @@
         <v>1</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>4</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="K1" s="2"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="B2" s="1">
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D2" s="1">
         <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>10</v>
+        <v>17</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="B3" s="1">
         <v>1</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="D3" s="1">
         <v>1</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="J3" s="1" t="s">
         <v>18</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>19</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
-  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>

</xml_diff>